<commit_message>
tune(girls): EXP 曲線 ×2.5＋標出三隻 boss ver -1027
Ray：「現在三女角升級太快了，以諾薇兒為例她在安雅登場前（娜塔莉戰前）差不多可以
      升到 lv2~lv3 是最妥當的。也就是訓練用聖徒、賞金獵人、蜈蚣（boss）、
      北泊掃盪(含一個 boss)、紫黑之爪(boss)後可以升到 lv3」

■ 校準方式：**照他點名的那條路實算**，不是憑感覺乘一個數
  · 訓練用聖徒＝教學戰，`tutorialSettle` **不發 EXP** → 0
  · 其餘四場各一局（北泊掃盪整段是一個 `session`，收段那一場才結算）
  · 蜈蚣／北泊收段（np_boss）／紫黑之爪三隻都是 boss（`bossMul.exp` ×2）
  實算（含 jitter）：55 分 4326／65 分 4956／75 分 5544／85 分 6160

■ `expTo` [0,600,1500,…,20000] → **×2.5** [0,1500,3800,7000,11500,17500,25500,36000,50000]
  ⇒ **55~85 分全部落在 Lv3**，過程是 賞金獵人 Lv1 → 蜈蚣 Lv2 → 北泊 Lv2 →
    **紫黑之爪 Lv3** —— 與「lv2~lv3」「紫黑之爪後 lv3」一字對得上。
  ⚠ 試過 ×3（低分會掉回 Lv2）與 ×3.5（要 75 分以上才 Lv3），都不夠穩。

■ 順帶把 Ray 在同一句裡點名的三隻標成 `boss:1`（-1024 是全部填 0 等他指定）：
  `centipi`（蜈蚣）／`np_boss`（北泊掃盪收段）／`np_claws`（紫黑之爪）。
  沒有這三個 1，boss ×2 不會生效，上面那條曲線也就對不上。

■ enemies.xlsx／girlstars.xlsx 重出。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/enemies.xlsx
+++ b/enemies.xlsx
@@ -4661,7 +4661,7 @@
         <v>1</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17" s="4" t="inlineStr"/>
       <c r="M17" s="4" t="inlineStr"/>
@@ -4822,7 +4822,7 @@
         <v>1</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" s="4" t="inlineStr"/>
       <c r="M18" s="4" t="inlineStr"/>
@@ -6112,7 +6112,7 @@
         <v>1</v>
       </c>
       <c r="K26" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L26" s="4" t="b">
         <v>1</v>
@@ -14362,7 +14362,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>74f847d6c9c55d02e1cdba6844bf55591bf098ad5e72e0a078d018fe3d3ea6f3</t>
+          <t>6af6db9db55fe35ef4c75bbfb7aa258c027b2e5e1fbfd79125f28905062bb97a</t>
         </is>
       </c>
     </row>

</xml_diff>